<commit_message>
Generate Soul v1.1-alpha templates
</commit_message>
<xml_diff>
--- a/financial-analyzer/test_runs/henglong_soul_contract/financial_output.xlsx
+++ b/financial-analyzer/test_runs/henglong_soul_contract/financial_output.xlsx
@@ -532,7 +532,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -619,7 +619,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>debt, liquidity, risk_management</t>
+          <t>debt, liquidity, restricted_assets</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>cash, debt, liquidity, risk_management</t>
+          <t>cash, debt, liquidity, restricted_assets, risk_management</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -765,7 +765,7 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
@@ -917,7 +917,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>debt, liquidity, risk_management, 银行贷款及其他借贷</t>
+          <t>debt, liquidity, restricted_assets, risk_management, 银行贷款及其他借贷</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -943,7 +943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1137,7 +1137,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>银行贷款及其他借贷</t>
+          <t>restricted_assets</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1149,6 +1149,26 @@
         </is>
       </c>
       <c r="D10" t="inlineStr">
+        <is>
+          <t># 17银行贷款及其他借贷 于结算日，无抵押银行贷款及其他借贷之还款期如下： 银行贷款（附注17(a)） 一年内或即期 一年后但二年内 二年后但五年内 26,351 22,468 五年以上 42,654 37,235 其他借贷（附注17(b)） 一年内或即期 970 一年后但二年内 二年后但五年内 五年以上 400 14,920 13,663 57,574 50,898 减：未摊销之财务费用 银…</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>银行贷款及其他借贷</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t># 17银行贷款及其他借贷 于结算日，无抵押银行贷款及其他借贷之还款期如下： 银行贷款（附注17(a)） 一年内或即期 一年后但二年内 二年后但五年内 26,351 22,468 五年以上 42,654 37,235 其他借贷（附注17(b)） 一年内或即期 970 一年后但二年内 二年后但五年内 五年以上 400 14,920 13,663 57,574 50,898 减：未摊销之财务费用 银…</t>
         </is>
@@ -1172,7 +1192,7 @@
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1455,7 +1475,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>适用于存在明显债务融资结构的发行人</t>
+          <t>适用于受限资金、抵押资产较多的地产或高杠杆主体</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1487,7 +1507,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>适用于存在明显债务融资结构的发行人</t>
+          <t>适用于受限资金、抵押资产较多的地产或高杠杆主体</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">

</xml_diff>